<commit_message>
Add the funding and resources playbook (PDF) and the 4-question investor table
Investor profiles cover stage, check size and lead/follow for the 103 A and B group
investors; the playbook walks through the Sophinos method and the resource catalogue.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V2WBTUaYVg19XogRfpJJ3d
</commit_message>
<xml_diff>
--- a/collateral/SimReal-投资人总表.xlsx
+++ b/collateral/SimReal-投资人总表.xlsx
@@ -542,17 +542,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>种子、A 轮</t>
+          <t>种子到成长期均投，A 轮为主</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>约 50 万–5000 万美元区间（聚合站数据）；种子首投具体额未确认</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>常领投 A 轮；种子轮领投比例未确认</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -604,17 +604,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>A 轮</t>
+          <t>pre-seed 到 A 轮，种子为主</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>种子约 25–200 万美元，甜蜜点约 50 万美元（聚合站数据）</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 0 次</t>
+          <t>近年多领投（Fund III 约 80–90% 为领投）</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -666,17 +666,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>B 轮及以后、种子</t>
+          <t>种子到 B 轮</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>早期约 25 万美元起；A 轮首投约 400–700 万美元（聚合站数据）</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>A 轮常领投（聚合站数据）；种子轮未确认</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -728,12 +728,12 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>早期为主（种子到 A 轮），少量成长期</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>50 万–1500 万美元，少数成长期可达 2500 万美元</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>A 轮、B 轮及以后、种子</t>
+          <t>种子到成长期全阶段</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -800,7 +800,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 4 次</t>
+          <t>常领投种子/A 轮</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -852,7 +852,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>种子、A 轮</t>
+          <t>种子到成长期，A 轮为主</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -862,7 +862,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 0 次</t>
+          <t>常领投 A 轮；种子轮未确认</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -914,7 +914,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>A 轮、种子</t>
+          <t>种子和 A 轮</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -924,7 +924,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>定位为领投种子/A 轮（高集中度投资）</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -976,17 +976,17 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>种子</t>
+          <t>种子到 A 轮为主，AI 原生公司</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>种子约 100–500 万美元；整体 100 万–2500 万美元（聚合站数据）</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>未确认</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -1038,17 +1038,17 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>种子</t>
+          <t>pre-seed 到种子+，种子为主</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>约 10 万–1000 万美元区间（聚合站数据）；种子具体额未确认</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>常领投种子（自称技术创始人的“第一张支票”）</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1100,17 +1100,17 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>未标明、A 轮</t>
+          <t>种子到成长期均投，近年大额以 A 轮后/成长期为主</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>约 25 万–5000 万美元（聚合站数据）</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 2 次</t>
+          <t>可领投（如 Infisical A 轮、Abridge D 轮）；种子轮多为跟投，比例未确认</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -1162,17 +1162,17 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>A 轮</t>
+          <t>pre-seed 到种子</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>pre-seed 10–50 万美元；种子 25–150 万美元，甜蜜点 30–80 万美元（聚合站数据）</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 0 次</t>
+          <t>未确认</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1224,17 +1224,17 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>种子、A 轮、B 轮及以后</t>
+          <t>种子到成长期全阶段，设有专门美国种子平台</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>种子约 200–1000 万美元（聚合站数据）</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 4 次</t>
+          <t>常领投种子/A 轮（如领投 Numos 425 万美元种子轮）</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>A 轮</t>
+          <t>未确认（官网称做成长期公司的战略投资，实际也投早期加密项目）</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1296,7 +1296,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 0 次</t>
+          <t>未确认</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1348,7 +1348,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>A 轮</t>
+          <t>早期到成长期全阶段（天使/A 轮到 Pre-IPO）</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -1358,7 +1358,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 0 次</t>
+          <t>未确认</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1410,7 +1410,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>种子</t>
+          <t>种子到 IPO 全阶段，种子和 A 轮为起点</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -1420,7 +1420,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 2 次</t>
+          <t>常领投种子/A 轮</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1472,7 +1472,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>未确认（公开案例为 Numerata 种子轮）</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1482,7 +1482,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>领投过 Numerata 种子轮（并成为其旗舰客户）</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -1534,7 +1534,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>B 轮及以后、A 轮、种子</t>
+          <t>种子和 A 轮为主（另有成长基金）</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1544,7 +1544,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>常领投种子/A 轮</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1596,7 +1596,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>种子、A 轮</t>
+          <t>种子为主</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 0 次</t>
+          <t>未确认</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1658,17 +1658,17 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>B 轮及以后、种子、A 轮</t>
+          <t>种子到成长期全阶段；AI 数据/基础设施方向种子、A 轮很活跃</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>未确认；参考：2026 年 5 月领投 Origin Lab 种子轮，整轮 800 万美元</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 3 次</t>
+          <t>常领投种子轮（如 Origin Lab 种子轮，由 Faraz Fatemi 领投）</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1720,17 +1720,17 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>种子、A 轮</t>
+          <t>Inception（pre-seed/种子）到成长期；2026 年 6 月新募 30 亿美元：Menlo XVII 投种子到 A 轮，Inflection IV 投 B 轮及以后</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>Inception/种子约 50–200 万美元（第三方数据库口径，非官方）；也做大额种子（领投 Inception Labs 5000 万美元种子）；Anthology Fund 起步约 10 万美元</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>种子/A 轮可领投（如 Inception Labs 种子轮）</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -1782,17 +1782,17 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>pre-seed/天使、A 轮</t>
+          <t>种子到成长期，近年聚焦人工智能</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>种子到 A 轮单笔 200–2000 万美元（公开披露口径）</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 0 次</t>
+          <t>未确认</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1844,17 +1844,17 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>A 轮</t>
+          <t>种子与 A 轮为主，聚焦企业级/AI 基础设施</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>种子约 100–300 万美元、A 轮约 300–800 万美元（第三方口径，非官方）；但领投的 Bespoke Labs A 轮整轮达 3180 万美元</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 2 次</t>
+          <t>常领投 A 轮（如 Bespoke Labs A 轮）</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -1906,7 +1906,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>A 轮及以前（天使为主），方向为 AI、机器人、硬件、航天</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1916,7 +1916,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>未确认（已知案例多为参投，如原力灵机 2 亿元天使轮）</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -1968,17 +1968,17 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>pre-seed/天使</t>
+          <t>早期为主（种子/天使/A 轮），后续多轮超配</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>未确认；参考：领投矩阵起源千万美元级天使轮</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>常领投早期轮次（如矩阵起源天使轮）</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -2030,7 +2030,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>早期到成长期（A、B 轮为主，也投天使）</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -2092,7 +2092,7 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>A 轮</t>
+          <t>早期为主（天使到 A 轮）</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -2102,7 +2102,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>未确认</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -2154,17 +2154,17 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>天使/种子为主，后续轮次跟进</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>未确认；历史案例天使/种子出资从数十万到约 1500 万人民币不等</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>天使轮常领投或独投（公开案例口径，未见官方表述）</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -2216,7 +2216,7 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>pre-seed/天使、未标明、A 轮</t>
+          <t>种子到成长期全阶段，2018 年设立种子基金</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -2226,7 +2226,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 2 次</t>
+          <t>未确认</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2278,7 +2278,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>pre-seed/天使</t>
+          <t>未确认（公开常识为技术驱动的早期投资）</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 0 次</t>
+          <t>未确认</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -2340,17 +2340,17 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>pre-seed/天使</t>
+          <t>早期兼顾成长期，首次投资多在 Pre-A 到 B 轮</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>未确认（已投近 3 亿美元、70 余个项目，平均约 400 万美元/项目，为推算值）</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 0 次</t>
+          <t>未确认</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -2392,27 +2392,27 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>天使</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>海外（未确认具体地区）</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>种子</t>
+          <t>种子/早期为主（个人天使）</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>未确认（数据库所列 100 万–1.2 亿美元实为整轮金额，不能代表个人支票）</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>多为跟投（个人天使，未确认）</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -2422,7 +2422,7 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>Balaji Srinivasan（本人，前 a16z 普通合伙人、前 Coinbase CTO）</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
@@ -2454,27 +2454,27 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>VC</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>海外（美国）</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>A 轮、B 轮及以后、种子、未标明</t>
+          <t>早期为主（A 轮为核心），也领投大额种子</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>未确认；参考：2025 年 6 月领投 Applied Compute 种子轮，整轮 2000 万美元（估值 1 亿美元）</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 3 次</t>
+          <t>常领投并进董事会（如 Applied Compute 种子轮）</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -2484,7 +2484,7 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>Victor Lazarte、Bill Gurley</t>
+          <t>Chetan Puttagunta（General Partner，基础设施/AI 方向）；备选 Everett Randle（General Partner，2025 年 10 月加入，AI 方向）</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
@@ -2516,17 +2516,17 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>VC</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>国内（上海）</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>未标明、A 轮</t>
+          <t>未确认；聚焦硬科技（半导体、高端装备、商业航天等），数据服务案例为博登智能 A+/A++ 轮</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -2536,7 +2536,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>未确认（博登智能 A+/A++ 轮为多家联合投资）</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -2546,7 +2546,7 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>应伟（管理合伙人，2012 年创建百孚）</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
@@ -2588,17 +2588,17 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>A 轮</t>
+          <t>种子到 A 轮早期</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>约 75–400 万美元（第三方口径，非官方）</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 0 次</t>
+          <t>未确认；Deeptune A 轮为跟投（a16z 领投）</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -2650,17 +2650,17 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>种子</t>
+          <t>种子为主</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>10 万到约 1000 万美元，最常见约 300 万美元；Fund III 平均单笔 300–500 万美元</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 0 次</t>
+          <t>未确认</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -2712,17 +2712,17 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>A 轮</t>
+          <t>早期到成长期，案例为 A 轮领投</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>未确认；参考：领投 AfterQuery A 轮，整轮 3000 万美元（投后 3 亿美元）</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>可领投 A 轮（如 AfterQuery）</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -2774,17 +2774,17 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>种子</t>
+          <t>pre-seed 到种子为主，偶尔跟进熟悉公司的 A 轮</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>约 25–200 万美元；常见 50–100 万美元（pre-seed 25–75 万，种子 50–100 万）</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 0 次</t>
+          <t>多为跟投（以共同投资为主，较少领投）</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -2836,17 +2836,17 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>种子、pre-seed/天使、未标明</t>
+          <t>种子到 B 轮，种子/初创期为主（2016–2020 年约 81% 的投资笔数）</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>第三方口径偏好单笔 100 万–5000 万人民币（自有表述未确认）</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>领投与跟投均有；如生数科技天使轮为跟投（蚂蚁领投），总体倾向未确认</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2898,12 +2898,12 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>种子到 A 轮</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>未确认（新基金 Deviation V 目标规模 3 亿美元）</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -2960,12 +2960,12 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>不限阶段，主投种子和 A 轮</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>首笔约 100 万–500 万美元以上（第三方数据库口径）</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -3022,7 +3022,7 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>种子</t>
+          <t>未确认（参与过 Mechanize 早期融资）</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -3032,7 +3032,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 0 次</t>
+          <t>未确认（个人天使通常不领投）</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -3084,7 +3084,7 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>A 轮、种子</t>
+          <t>早期（个人天使组合约 3 家，含 Positron、Prime Intellect）</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -3094,7 +3094,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 0 次</t>
+          <t>未确认（个人天使通常不领投）</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -3146,17 +3146,17 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>种子</t>
+          <t>pre-seed 到种子，种子为主（不投 A 轮以后）</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>首笔约 35 万–300 万美元，平均 125–150 万美元（官网）；Eniac V 口径为 50–500 万美元，平均 150–200 万美元</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 0 次</t>
+          <t>常领投或联合领投种子轮（每位 GP 每年领投 2–3 家）</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -3208,17 +3208,17 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>种子为主</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>未确认（领投的 Poindexter Labs 种子轮总额 200 万英镑；Tracxn 统计其种子轮平均轮次规模约 285 万美元）</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>可领投种子轮（如领投 Poindexter Labs）</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -3270,17 +3270,17 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>种子</t>
+          <t>种子到 A 轮为主，也做后续轮次</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>约 10 万–500 万美元；种子/A 轮估计 25 万–200 万美元以上（第三方口径）</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 0 次</t>
+          <t>领投与跟投均有（如 2025 年 11 月领投 Aily Labs 8000 万美元 B 轮）；种子/A 轮倾向未确认</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -3332,17 +3332,17 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>种子</t>
+          <t>pre-seed 到 A 轮</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>约 50–500 万美元</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>常领投种子轮（如 2026 年 1 月领投 AgileRL 750 万美元种子轮）</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -3394,17 +3394,17 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>种子、A 轮</t>
+          <t>pre-seed 到 B 轮</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>个人支票约 2.5–100 万美元（第三方口径，未经本人确认）</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 0 次</t>
+          <t>多为跟投</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -3456,17 +3456,17 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>种子</t>
+          <t>pre-seed 到 A 轮，种子为主</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>种子约 100–500 万美元，pre-seed 75–250 万美元（第三方口径）</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 0 次</t>
+          <t>常领投或联合领投种子轮（如领投 Mage 630 万美元种子轮）；A 轮较少领投</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -3518,17 +3518,17 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>pre-seed 和种子为主（约 90%），也跟进 A 轮及以后</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>平均约 100 万美元，范围约 20 万–200 万美元（Hunter Walk 访谈）</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>可领投种子轮，也常作为参与方</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -3580,7 +3580,7 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>A 轮</t>
+          <t>未确认</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -3590,7 +3590,7 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 0 次</t>
+          <t>未确认（个人天使通常不领投）</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -3642,17 +3642,17 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>pre-seed 到 A 轮，A 轮为主</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>约 100–1500 万美元；A 轮 300–1500 万美元</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>A 轮常领投；种子轮倾向未确认</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -3704,17 +3704,17 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>种子</t>
+          <t>pre-seed 和种子为主</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>约 10–300 万美元，平均 25–200 万美元</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>常作为首个机构投资方或领投方（第三方口径）</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -3766,12 +3766,12 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>种子到成熟期均投</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>未确认（历史单笔从数十万到亿元级人民币不等）</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -3828,17 +3828,17 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>未标明</t>
+          <t>不限阶段，种子到成长期</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>早期（pre-seed/种子）约 10 万–1000 万美元；Grace Isford 投资区间约 50 万–5000 万美元（第三方口径）</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>常领投或联合领投（Grace Isford 近期领投或联合领投多笔 AI 基础设施种子轮）</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
@@ -3890,17 +3890,17 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>A 轮</t>
+          <t>pre-seed 到 B 轮，种子和 A 轮为主</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>第三方数据库：首张支票约 100–1000 万美元，种子轮常领投 300–600 万美元</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>常领投种子轮和 A 轮</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3952,17 +3952,17 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>A 轮</t>
+          <t>从成立初期（inception）到种子、A 轮；AI Start 基金专做 AI 种子</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>AI Start 种子基金（2023 年 2.5 亿美元）典型支票 100–400 万美元</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 0 次</t>
+          <t>多为领投/联合领投（Mayfield 惯例；AI Start 领投比例未确认）</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4014,17 +4014,17 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>种子、A 轮</t>
+          <t>pre-seed 到 A 轮，pre-seed 和种子为主</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>pre-seed 约 25–200 万美元；种子约 100–600 万美元（第三方汇总）</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 0 次</t>
+          <t>常领投/联合领投 pre-seed 与种子轮（PearX 项目领投 pre-seed）</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
@@ -4076,17 +4076,17 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>pre-seed 到 pre-IPO，种子和 A 轮为主</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>第三方数据库：种子约 25–200 万美元，A 轮约 200–1500 万美元</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>领投与跟投均有（比例未确认）</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
@@ -4138,17 +4138,17 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>种子</t>
+          <t>种子到成长期；早期基金专注种子和 A 轮</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>第三方数据库：种子约 50–200 万美元、A 轮约 200–800 万美元（实际 A 轮常更大）；第十期早期基金 6.5 亿美元（2025 年 5 月）</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>A 轮常领投；种子领投与跟投均有（与 Sequoia 联合领投 Irregular）</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
@@ -4200,17 +4200,17 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>pre-seed 与种子为主</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>首张支票约 75–150 万美元（早期基金为 25–50 万美元）</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>多为联合投资/跟投，刻意与其他机构共同投；偶尔领投（如 Proximal）</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
@@ -4262,17 +4262,17 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>种子、A 轮、未标明、B 轮及以后</t>
+          <t>pre-seed 到成长期全阶段；Arc 项目做 pre-seed/种子</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>Arc 首张支票约 50–100 万美元；常规种子/A 轮支票未确认（2025 年新募 2 亿美元种子基金 + 7.5 亿美元 A 轮基金）</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 5 次</t>
+          <t>常领投种子和 A 轮（如领投 Irregular）；Arc 本身不领投后续种子轮</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
@@ -4324,7 +4324,7 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>种子</t>
+          <t>天使/种子</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
@@ -4334,7 +4334,7 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 0 次</t>
+          <t>多为跟投（个人天使）</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
@@ -4386,17 +4386,17 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>A 轮</t>
+          <t>只做 A 轮（post-PMF 公司）</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>单笔约 500–1000 万美元，固定约 10% 稀释，不要董事会席位；Fund I 4.25 亿美元</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>领投 A 轮</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
@@ -4448,17 +4448,17 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>种子、A 轮</t>
+          <t>种子为主</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>种子基金通常约 20 万美元</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>不领投，通常为轮次中的较小跟投支票</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
@@ -4510,17 +4510,17 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>A 轮</t>
+          <t>种子到成长期（通过 Raine Ventures）</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>第三方数据库：早期支票约 100–1500 万美元</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 0 次</t>
+          <t>多为跟投（如参投 Altos 领投的 AfterQuery A 轮）</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
@@ -4572,17 +4572,17 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>孵化、pre-seed 和种子</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>约 25–300 万美元</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>未确认（以孵化/种子为主，领投比例未知）</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
@@ -4634,17 +4634,17 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>种子</t>
+          <t>pre-seed 与种子</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>约 25 万美元起（Fund I 4500 万美元，两年内投约 80 家）</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 0 次</t>
+          <t>推断多为跟投（基金规模小、投资数量多，未确认）</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
@@ -4696,7 +4696,7 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>A 轮</t>
+          <t>天使/种子</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
@@ -4706,7 +4706,7 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 0 次</t>
+          <t>多为跟投（个人天使）</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
@@ -4758,7 +4758,7 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>pre-seed/天使</t>
+          <t>传统以成长期为主，近期也参与天使轮（如 TalentsAI）</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
@@ -4768,7 +4768,7 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 0 次</t>
+          <t>未确认（TalentsAI 天使轮为参投）</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
@@ -4820,17 +4820,17 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>种子、天使、A 轮为主，B 轮选择性跟投</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>未确认（领投硅基流动 5000 万元人民币天使轮，为整轮金额）</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>常领投天使/早期轮（如领投硅基流动天使轮，A 轮老股东超额跟投）</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
@@ -4882,17 +4882,17 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>A 轮</t>
+          <t>以 A、B 轮为主，向早期和中后期延伸</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>未确认（领投星尘数据 5000 万元人民币 A 轮，为整轮金额）</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>A、B 轮常领投</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
@@ -4944,17 +4944,17 @@
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>初创期、成长期、扩张期均投（早期及成长期人民币基金）</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>未确认（单笔金额未公开）</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>领投与联合领投常见（与启明创投联合领投智谱 1 亿元 B 轮，并持续加注）</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
@@ -5006,7 +5006,7 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>未标明、B 轮及以后、pre-seed/天使</t>
+          <t>未确认；已知参与光轮智能 10 亿元 A++/A+++ 轮（偏中后期），种子/天使投资记录未查到</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
@@ -5016,7 +5016,7 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>在光轮智能该轮为参投的财务投资机构之一；领投习惯未确认</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
@@ -5068,17 +5068,17 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>未标明</t>
+          <t>未确认；已知联合领投恺望数据逾亿元战略轮（2026 年 8 月，公司已过 Pre-A）</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>未确认（恺望数据该轮总额逾亿元人民币，由三家联合领投）</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>可联合领投（恺望数据战略轮与亦庄产业基金、华方资本联合领投）</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
@@ -5130,7 +5130,7 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>天使到 A 轮早期为主（2026 年仍活跃于 AI 天使轮）</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
@@ -5140,7 +5140,7 @@
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>常领投或与红杉中国种子基金等联合投资天使轮（如 2026 年 ACONTEXT 天使轮、Catnip）</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
@@ -5192,17 +5192,17 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>A 轮</t>
+          <t>天使到成长期，早期（Pre-A/A 轮）为主</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>未确认（光轮智能 Pre-A 轮总额数千万人民币，由经纬领投）</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>常领投早期轮，并在后续轮超额跟投（光轮智能 Pre-A 领投、Pre-A+ 超额跟投，为最大机构股东）</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
@@ -5254,7 +5254,7 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>pre-seed/天使</t>
+          <t>早期为主（已知投资智能知识天使轮）</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 0 次</t>
+          <t>智能知识天使轮与锦秋基金联合投资；领投/跟投习惯未确认</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">
@@ -5316,7 +5316,7 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>天使到 A 轮早期为主（2026 年 4 月新募 39 亿元人民币，为当年最大早期募资）</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
@@ -5326,7 +5326,7 @@
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>未确认（2026 年一季度至少 7 起融资，多为早期；是否以领投为主本次未逐笔核实）</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
@@ -5378,17 +5378,17 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>pre-seed/天使</t>
+          <t>早期到成长期；已知领投 GIM 天使+轮</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>未确认（GIM 天使轮与天使+轮合计过亿元人民币）</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>可领投天使轮（领投 GIM 天使+轮）</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
@@ -5440,7 +5440,7 @@
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>种子</t>
+          <t>早期为主（天使到 A/B 轮），并在后续轮次追加（如世航智能 A 轮老股东追投）</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
@@ -5450,7 +5450,7 @@
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>未确认（广为报道以早期领投见长，本次未逐笔核实）</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr">
@@ -5502,7 +5502,7 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>pre-seed/天使、未标明</t>
+          <t>天使到成长期，近年 AI/机器人方向天使+ 到 A/B 轮均有出手</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
@@ -5512,7 +5512,7 @@
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>可联合领投（2026 年 6 月与锦秋基金联合领投聚能天擎数亿元天使+轮）；其余多为参投</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
@@ -5554,27 +5554,27 @@
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>VC</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>海外（印度，孟买）</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>A 轮</t>
+          <t>成长期为主（A 轮后段及以后），不以种子为主</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>未确认（领投 Deccan AI 2,500 万美元 A 轮，该轮另有 SIG、Prosus 参与）</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>常领投（成长期）；种子轮基本不参与</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5616,27 +5616,27 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>天使</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>海外（美国）</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>种子、未标明</t>
+          <t>种子/早期（个人天使，约 62 笔投资，偏应用 AI、开发者工具）</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>未确认（个人天使支票，金额未公开）</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 0 次</t>
+          <t>多为跟投（如 Patronus AI 种子轮由 Lightspeed 领投，其为参投天使）</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -5646,7 +5646,7 @@
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>Amjad Masad 本人（Replit 创始人兼 CEO）</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr">
@@ -5678,17 +5678,17 @@
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>VC</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>海外（美国，全球多地设点）</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>A 轮</t>
+          <t>早期到成长期（2022 年设 2.5 亿美元早期基金 Ascent Fund）；GIM 为 A 轮出手</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
@@ -5698,7 +5698,7 @@
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>可联合领投 A 轮（与金涌投资联合领投 GIM A 轮）；种子阶段领投习惯未确认</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr">
@@ -5708,7 +5708,7 @@
       </c>
       <c r="I85" s="2" t="inlineStr">
         <is>
-          <t>Howard Morgan</t>
+          <t>Howard Morgan（Chair 兼 General Partner；文艺复兴科技联合创始人、First Round Capital 联合创始人）</t>
         </is>
       </c>
       <c r="J85" s="2" t="inlineStr">
@@ -5740,27 +5740,27 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>VC</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>海外（美国）</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>种子</t>
+          <t>种子为主（加密/去中心化 AI 方向）；其他阶段未确认</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>未确认（与 Distributed Global 联合领投 Prime Intellect 550 万美元种子轮）</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>可联合领投种子轮（Prime Intellect）</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
@@ -5802,27 +5802,27 @@
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>VC</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>海外（美国，纽约）</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>pre-seed/天使、种子</t>
+          <t>pre-seed 到种子</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>未确认（AgileRL pre-seed 总额 150 万英镑，与 Octopus Ventures 联合领投）</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>可联合领投 pre-seed，并在种子轮跟投（AgileRL）</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr">
@@ -5832,7 +5832,7 @@
       </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>Evan Burnstein（Partner，专注数据、AI 与基础设施的 pre-seed/种子投资，任 AgileRL 董事）</t>
         </is>
       </c>
       <c r="J87" s="2" t="inlineStr">
@@ -5864,27 +5864,27 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>VC</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>海外（未确认）</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>种子</t>
+          <t>种子（已知）；其他阶段未确认</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>未确认（与 CoinFund 联合领投 Prime Intellect 550 万美元种子轮）</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>可联合领投种子轮（Prime Intellect）</t>
         </is>
       </c>
       <c r="H88" s="2" t="inlineStr">
@@ -5926,27 +5926,27 @@
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>VC</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>海外（美国）</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>种子、B 轮及以后</t>
+          <t>种子到 A 轮为主，主打首轮机构支票</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>约 25 万–1,500 万美元，平均 100–1,000 万美元（第三方目录数据）；领投 Turing 1,400 万美元种子轮</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>常领投种子轮（Turing 种子轮由 Ashu Garg 领投）</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr">
@@ -5956,7 +5956,7 @@
       </c>
       <c r="I89" s="2" t="inlineStr">
         <is>
-          <t>Ashu Garg</t>
+          <t>Ashu Garg（General Partner，专投深度技术 AI 创始人的首轮支票，Turing 董事）</t>
         </is>
       </c>
       <c r="J89" s="2" t="inlineStr">
@@ -5988,27 +5988,27 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>VC</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>海外（美国）</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>种子</t>
+          <t>种子到成长期全阶段</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>未确认（领投 Prime Intellect 1,500 万美元种子延期轮）</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>常领投（领投 Prime Intellect 2025 年 2 月轮次）</t>
         </is>
       </c>
       <c r="H90" s="2" t="inlineStr">
@@ -6050,27 +6050,27 @@
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>VC</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>海外（加拿大）</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>种子</t>
+          <t>种子起投（与 General Catalyst 联合领投 Good Start Labs 种子轮）；后期阶段未在本次检索中核实</t>
         </is>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>未确认（Good Start Labs 种子轮总额 360 万美元）</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>可联合领投种子轮（Good Start Labs，2025 年 10 月）</t>
         </is>
       </c>
       <c r="H91" s="2" t="inlineStr">
@@ -6112,27 +6112,27 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>VC</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>海外（美国，硅谷/旧金山/纽约）</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>A 轮、B 轮及以后</t>
+          <t>种子到 A 轮为主，也做 B 轮及成长期</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>种子起步约 50 万美元；A/B 轮甜区约 1500–2000 万美元（第三方汇总，未经基金官方确认）</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>常领投 A 轮（领投 Patronus AI 1700 万美元 A 轮，Glenn Solomon 入董事会）；种子轮是否常领投未确认</t>
         </is>
       </c>
       <c r="H92" s="2" t="inlineStr">
@@ -6142,7 +6142,7 @@
       </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>Glenn Solomon</t>
+          <t>Glenn Solomon（Managing Partner，主导 Patronus AI A 轮并入董事会）</t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr">
@@ -6174,27 +6174,27 @@
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>VC</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>海外（美国，康涅狄格州格林威治）</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>A 轮</t>
+          <t>种子到成长期，专注金融科技和医疗；金融科技方向以 A 轮及之后为主</t>
         </is>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>第三方汇总为 100 万–1 亿美元；领投 Halluminate 3000 万美元 A 轮；据报道 2026 年 3 月 Fund VI 募资近 20 亿美元</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>常领投 A 轮及之后（领投 Halluminate A 轮）；种子轮领投频率未确认</t>
         </is>
       </c>
       <c r="H93" s="2" t="inlineStr">
@@ -6204,7 +6204,7 @@
       </c>
       <c r="I93" s="2" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>Matt Streisfeld（General Partner，金融科技方向，主导 Halluminate A 轮）</t>
         </is>
       </c>
       <c r="J93" s="2" t="inlineStr">
@@ -6236,27 +6236,27 @@
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>VC</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>海外（英国，伦敦）</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>pre-seed/天使、种子</t>
+          <t>pre-seed 到 A 轮切入，后续跟到 B 轮及以后</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>pre-seed 约 10–75 万英镑（标准约 10 万英镑）；种子/A 轮约 100 万英镑起；第三方称平均单笔约 450 万英镑</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>pre-seed 阶段可领投（深科技 pre-seed 基金定位为领投方）；在 AgileRL 中为跟投（种子轮由 Fusion Fund 领投）</t>
         </is>
       </c>
       <c r="H94" s="2" t="inlineStr">
@@ -6298,27 +6298,27 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>VC</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>海外（美国，旧金山）</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>种子、A 轮</t>
+          <t>YC 批次期 pre-seed/种子，后续轮次会跟投（如 Halluminate A 轮）</t>
         </is>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>未确认（基金约 4000 万美元，自 2023 年冬季批次起已投 116 家 YC 公司；自称少投多下注）</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 0 次</t>
+          <t>多为跟投</t>
         </is>
       </c>
       <c r="H95" s="2" t="inlineStr">
@@ -6328,7 +6328,7 @@
       </c>
       <c r="I95" s="2" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>Dave Yen / Jason Freedman（联合创始人）</t>
         </is>
       </c>
       <c r="J95" s="2" t="inlineStr">
@@ -6360,27 +6360,27 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>VC</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>国内（城市未确认）</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>A 轮、未标明</t>
+          <t>未确认（领投过恺望数据 Pre-A 轮）</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>未确认（恺望数据 Pre-A 轮总额为数千万元人民币，亚盛领投）</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>领投过恺望数据 Pre-A 轮；是否常领投未确认</t>
         </is>
       </c>
       <c r="H96" s="2" t="inlineStr">
@@ -6422,27 +6422,27 @@
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>VC</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>国内（城市未确认）</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>pre-seed/天使</t>
+          <t>天使轮（与东方富海联合领投枢途科技天使轮）；整体偏好未确认</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>未确认（枢途科技天使轮总额为数千万元人民币）</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>联合领投过枢途科技天使轮；是否常领投未确认</t>
         </is>
       </c>
       <c r="H97" s="2" t="inlineStr">
@@ -6484,27 +6484,27 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>天使</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>国内（杭州）</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>pre-seed/天使</t>
+          <t>天使/种子为主</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>未确认（星尘数据天使轮总额为数百万元人民币，天使湾领投）</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>常领投天使轮（领投星尘数据天使轮，英诺天使等跟投）</t>
         </is>
       </c>
       <c r="H98" s="2" t="inlineStr">
@@ -6546,27 +6546,27 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>战略投资</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>国内（深圳）</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>A 轮、pre-seed/天使</t>
+          <t>全阶段战略投资，AI 方向多为中后期大额轮次</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>未确认（参与 UniPat 3 亿美元融资，估值 25 亿美元，腾讯份额未披露）</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 0 次</t>
+          <t>多为跟投（UniPat 轮由阿里领投，腾讯参与）</t>
         </is>
       </c>
       <c r="H99" s="2" t="inlineStr">
@@ -6608,17 +6608,17 @@
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>战略投资</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>国内（深圳）</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>种子</t>
+          <t>早期产业投资（领投简智机器人种子+轮）</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
@@ -6628,7 +6628,7 @@
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>领投过简智机器人种子+轮（百度风投跟投）；是否常领投未确认</t>
         </is>
       </c>
       <c r="H100" s="2" t="inlineStr">
@@ -6638,7 +6638,7 @@
       </c>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>邱纯潮（CEO，曾公开评价对简智的投资）</t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr">
@@ -6670,27 +6670,27 @@
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>战略投资</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>中国香港（港股上市平台）</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>A 轮</t>
+          <t>A 轮（联合领投 GIM A 轮）；整体偏好未确认</t>
         </is>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>GIM A 轮投资 650 万美元（单一案例）</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>联合领投 GIM A 轮（与 B Capital 一起）并进入董事会</t>
         </is>
       </c>
       <c r="H101" s="2" t="inlineStr">
@@ -6732,27 +6732,27 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>VC</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>国内（杭州）</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>pre-seed/天使</t>
+          <t>未确认（领投过心识宇宙天使+轮）</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>未确认（心识宇宙天使和天使+两轮合计近亿元人民币）</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>领投过心识宇宙天使+轮；是否常领投未确认</t>
         </is>
       </c>
       <c r="H102" s="2" t="inlineStr">
@@ -6762,7 +6762,7 @@
       </c>
       <c r="I102" s="2" t="inlineStr">
         <is>
-          <t>未找到</t>
+          <t>陈向明（创始人，公开评价过心识宇宙投资）</t>
         </is>
       </c>
       <c r="J102" s="2" t="inlineStr">
@@ -6794,27 +6794,27 @@
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>战略投资</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>国内（杭州）</t>
         </is>
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>A 轮</t>
+          <t>战略/成长期大额轮次为主</t>
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>未确认（领投 UniPat 3 亿美元轮，估值 25 亿美元，阿里出资份额未披露）</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>领投 UniPat 轮</t>
         </is>
       </c>
       <c r="H103" s="2" t="inlineStr">
@@ -6856,27 +6856,27 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>国内（城市未确认）</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>A 轮</t>
+          <t>Pre-A（联合领投枢途科技 Pre-A 轮）；整体偏好未确认</t>
         </is>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>未确认</t>
+          <t>未确认（枢途科技 Pre-A 轮总额近亿元人民币，与鼎晖百孚联合领投）</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t>同类公司中领投 1 次</t>
+          <t>联合领投过枢途科技 Pre-A 轮；是否常领投未确认</t>
         </is>
       </c>
       <c r="H104" s="2" t="inlineStr">

</xml_diff>